<commit_message>
WIP: hourly save 2026-09-28T04:38:09.4281430-04:00
</commit_message>
<xml_diff>
--- a/data/GuildRule.xlsx
+++ b/data/GuildRule.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +452,25 @@
           <t>reunion_min_online_members</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>activity_join_min_hours</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>trial_invite_ttl_seconds</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>trial_invite_cooldown_seconds</t>
+        </is>
+      </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
@@ -487,6 +505,21 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>中秋团圆在线人数兜底阈值(B6a 读取)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>参与帮会活动所需最短入帮时长(小时,B6a 读取),0-720</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>同道历练邀请房间有效期(秒,B6b 读取),10-120</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>同一发起人两次成功建历练房间的最小间隔(秒,B6b 读取),0-600</t>
         </is>
       </c>
     </row>
@@ -511,6 +544,15 @@
       </c>
       <c r="G6" t="n">
         <v>3</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>30</v>
+      </c>
+      <c r="J6" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>